<commit_message>
Live auction states for screen cases; case routing by setup
Synced from procol-qa-platform e5a9ea0.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/procol test/fixtures/vendor-bulk-upload/VBU-120.xlsx
+++ b/procol test/fixtures/vendor-bulk-upload/VBU-120.xlsx
@@ -514,12 +514,6 @@
       <c r="M4" t="str">
         <v>400001</v>
       </c>
-      <c r="N4" t="str">
-        <v>QA Second Contact</v>
-      </c>
-      <c r="O4" t="str">
-        <v>qa_vbu_{{stamp}}_120_2@example.com</v>
-      </c>
       <c r="R4" t="str">
         <v>ZCOV</v>
       </c>

</xml_diff>